<commit_message>
Super Red LED trim target
</commit_message>
<xml_diff>
--- a/SAL_JIG/SAL_JIG_CS1/측정자료/sal_cs_2차샘플_전류trim_디버깅_250613.xlsx
+++ b/SAL_JIG/SAL_JIG_CS1/측정자료/sal_cs_2차샘플_전류trim_디버깅_250613.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oio95\OneDrive\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\Jig\SAL_JIG\SAL_JIG_CS1\측정자료\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B19E73-13D7-4321-9884-7FE19A3CB8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B93FD4-1C25-474B-82B4-14C8539AEAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="10515" windowWidth="29040" windowHeight="15720" xr2:uid="{254A9F07-DF4E-4845-91F9-FA135E5CFC76}"/>
+    <workbookView xWindow="9630" yWindow="0" windowWidth="19170" windowHeight="15480" xr2:uid="{254A9F07-DF4E-4845-91F9-FA135E5CFC76}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>CCC</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -51,6 +51,46 @@
   </si>
   <si>
     <t>2차</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CS Super Red</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>R</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>G</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>B</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>max current</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F123</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>After Trim</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Taregt</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -101,7 +141,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -110,6 +150,9 @@
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,18 +488,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF6510CE-E367-4981-AD5C-A302D6F7EA40}">
-  <dimension ref="B1:K9"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="B1:K26"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2">
         <v>14.284000000000001</v>
       </c>
@@ -472,7 +515,7 @@
         <v>3276</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>11.6</v>
       </c>
@@ -488,7 +531,7 @@
         <v>4095</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>5.4320000000000004</v>
       </c>
@@ -501,12 +544,12 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>15.715</v>
       </c>
@@ -519,7 +562,7 @@
         <v>15.714999999999996</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>11.6</v>
       </c>
@@ -532,7 +575,7 @@
         <v>11.599999999999998</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>5.9589999999999996</v>
       </c>
@@ -543,6 +586,191 @@
       <c r="E9">
         <f t="shared" si="2"/>
         <v>5.9589999999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>20</v>
+      </c>
+      <c r="F17">
+        <v>20</v>
+      </c>
+      <c r="G17">
+        <v>4095</v>
+      </c>
+      <c r="H17" t="str">
+        <f>_xlfn.CONCAT("0x", DEC2HEX(G17))</f>
+        <v>0xFFF</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>15.78</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18">
+        <v>15</v>
+      </c>
+      <c r="F18">
+        <v>15</v>
+      </c>
+      <c r="G18">
+        <v>4095</v>
+      </c>
+      <c r="H18" t="str">
+        <f t="shared" ref="H18:H19" si="3">_xlfn.CONCAT("0x", DEC2HEX(G18))</f>
+        <v>0xFFF</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19">
+        <v>10.050000000000001</v>
+      </c>
+      <c r="D19" s="3">
+        <v>6</v>
+      </c>
+      <c r="E19">
+        <v>10</v>
+      </c>
+      <c r="F19">
+        <v>10</v>
+      </c>
+      <c r="G19">
+        <v>4095</v>
+      </c>
+      <c r="H19" t="str">
+        <f t="shared" si="3"/>
+        <v>0xFFF</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24">
+        <v>20</v>
+      </c>
+      <c r="F24">
+        <v>16</v>
+      </c>
+      <c r="G24">
+        <f>ROUND(F24/E24*4095, 0)</f>
+        <v>3276</v>
+      </c>
+      <c r="H24" t="str">
+        <f>_xlfn.CONCAT("0x", DEC2HEX(G24))</f>
+        <v>0xCCC</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25">
+        <v>15.78</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25">
+        <v>15</v>
+      </c>
+      <c r="F25">
+        <v>13.82</v>
+      </c>
+      <c r="G25">
+        <f t="shared" ref="G25:G26" si="4">ROUND(F25/E25*4095, 0)</f>
+        <v>3773</v>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" ref="H25:H26" si="5">_xlfn.CONCAT("0x", DEC2HEX(G25))</f>
+        <v>0xEBD</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26">
+        <v>10.050000000000001</v>
+      </c>
+      <c r="D26" s="3">
+        <v>6</v>
+      </c>
+      <c r="E26">
+        <v>10</v>
+      </c>
+      <c r="F26">
+        <v>7.69</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="4"/>
+        <v>3149</v>
+      </c>
+      <c r="H26" t="str">
+        <f t="shared" si="5"/>
+        <v>0xC4D</v>
       </c>
     </row>
   </sheetData>

</xml_diff>